<commit_message>
Sync full project state: API/DB-optional data sources, UI validation stage, qaprod env, docs
- General Voucher API models, API-backed data sources and DB availability gating
- Common UI validation stage and specs for GV/AP/AR, plus unit tests
- New qaprod environment config and data workbooks
- Updated Jenkinsfile, TestNG suites and docs
- .gitignore: exclude local IDE data sources, generated graphify cache, logs and test-output

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/test/resources/env/staging/data/UsersList.xlsx
+++ b/src/test/resources/env/staging/data/UsersList.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7500"/>
+    <workbookView windowWidth="20370" windowHeight="8520"/>
   </bookViews>
   <sheets>
     <sheet name="UIUsers" sheetId="1" r:id="rId1"/>
@@ -1317,7 +1317,7 @@
         <v>5</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:2">

</xml_diff>